<commit_message>
Add 30-day progress and tools-used workbook details
</commit_message>
<xml_diff>
--- a/12pm_office_work_inventory.xlsx
+++ b/12pm_office_work_inventory.xlsx
@@ -2,7 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cyber Guardian" sheetId="1" r:id="Rc664420601794952"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cyber Guardian" sheetId="1" r:id="R376dc100d7e04f8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30-Day Progress" sheetId="2" r:id="R75ed05c9370e4ea0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tools Used" sheetId="3" r:id="R6acc39e50ef34dac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="3">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -30,13 +32,34 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -91,7 +114,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="21">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -100,6 +123,31 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -494,4 +542,717 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="58" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="44" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="9" t="str">
+        <x:v>Amala Cybersecurity Portfolio — 30-Day Progress</x:v>
+      </x:c>
+      <x:c r="B1" s="9" t="str"/>
+      <x:c r="C1" s="9" t="str"/>
+      <x:c r="D1" s="9" t="str"/>
+      <x:c r="E1" s="9" t="str"/>
+      <x:c r="F1" s="9" t="str"/>
+      <x:c r="G1" s="9" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="18" t="str">
+        <x:v>Day</x:v>
+      </x:c>
+      <x:c r="B3" s="18" t="str">
+        <x:v>Project</x:v>
+      </x:c>
+      <x:c r="C3" s="18" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="D3" s="18" t="str">
+        <x:v>Files / Evidence</x:v>
+      </x:c>
+      <x:c r="E3" s="18" t="str">
+        <x:v>Tests</x:v>
+      </x:c>
+      <x:c r="F3" s="18" t="str">
+        <x:v>Tools</x:v>
+      </x:c>
+      <x:c r="G3" s="18" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="19" t="str">
+        <x:v>Verify environment and create safe local lab</x:v>
+      </x:c>
+      <x:c r="C4" s="19" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D4" s="19" t="str">
+        <x:v>Day-01-Lab-Setup/README.md; src/verify_environment.py; tests/test_environment.py; evidence/environment-check.json</x:v>
+      </x:c>
+      <x:c r="E4" s="19" t="str">
+        <x:v>PASS: verifier; PASS: 1 unit test; NOT RUN: network scans</x:v>
+      </x:c>
+      <x:c r="F4" s="19" t="str">
+        <x:v>Python 3.13.14; Git 2.55.0; Ollama qwen3:4b; curl 8.21.0; PowerShell; OpenClaw</x:v>
+      </x:c>
+      <x:c r="G4" s="19" t="str">
+        <x:v>Initial path bug fixed and retested</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="19" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="19" t="str">
+        <x:v>Python security toolkit</x:v>
+      </x:c>
+      <x:c r="C5" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D5" s="19" t="str"/>
+      <x:c r="E5" s="19" t="str"/>
+      <x:c r="F5" s="19" t="str"/>
+      <x:c r="G5" s="19" t="str">
+        <x:v>Next project</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="19" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="19" t="str">
+        <x:v>Password-strength analyzer</x:v>
+      </x:c>
+      <x:c r="C6" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D6" s="19" t="str"/>
+      <x:c r="E6" s="19" t="str"/>
+      <x:c r="F6" s="19" t="str"/>
+      <x:c r="G6" s="19" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="19" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="19" t="str">
+        <x:v>Phishing URL heuristic detector</x:v>
+      </x:c>
+      <x:c r="C7" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D7" s="19" t="str"/>
+      <x:c r="E7" s="19" t="str"/>
+      <x:c r="F7" s="19" t="str"/>
+      <x:c r="G7" s="19" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="19" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="str">
+        <x:v>HTTP security-header checker</x:v>
+      </x:c>
+      <x:c r="C8" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D8" s="19" t="str"/>
+      <x:c r="E8" s="19" t="str"/>
+      <x:c r="F8" s="19" t="str"/>
+      <x:c r="G8" s="19" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="19" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="19" t="str">
+        <x:v>TLS certificate checker</x:v>
+      </x:c>
+      <x:c r="C9" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D9" s="19" t="str"/>
+      <x:c r="E9" s="19" t="str"/>
+      <x:c r="F9" s="19" t="str"/>
+      <x:c r="G9" s="19" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="19" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="19" t="str">
+        <x:v>Uptime and broken-link monitor</x:v>
+      </x:c>
+      <x:c r="C10" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D10" s="19" t="str"/>
+      <x:c r="E10" s="19" t="str"/>
+      <x:c r="F10" s="19" t="str"/>
+      <x:c r="G10" s="19" t="str"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="19" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="19" t="str">
+        <x:v>Dependency audit</x:v>
+      </x:c>
+      <x:c r="C11" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D11" s="19" t="str"/>
+      <x:c r="E11" s="19" t="str"/>
+      <x:c r="F11" s="19" t="str"/>
+      <x:c r="G11" s="19" t="str"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="19" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="str">
+        <x:v>Static analysis</x:v>
+      </x:c>
+      <x:c r="C12" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D12" s="19" t="str"/>
+      <x:c r="E12" s="19" t="str"/>
+      <x:c r="F12" s="19" t="str"/>
+      <x:c r="G12" s="19" t="str"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="19" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="19" t="str">
+        <x:v>Secure input validation</x:v>
+      </x:c>
+      <x:c r="C13" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D13" s="19" t="str"/>
+      <x:c r="E13" s="19" t="str"/>
+      <x:c r="F13" s="19" t="str"/>
+      <x:c r="G13" s="19" t="str"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="19" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B14" s="19" t="str">
+        <x:v>SQL injection training lab</x:v>
+      </x:c>
+      <x:c r="C14" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D14" s="19" t="str"/>
+      <x:c r="E14" s="19" t="str"/>
+      <x:c r="F14" s="19" t="str"/>
+      <x:c r="G14" s="19" t="str">
+        <x:v>Local lab only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="19" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="19" t="str">
+        <x:v>XSS prevention training lab</x:v>
+      </x:c>
+      <x:c r="C15" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D15" s="19" t="str"/>
+      <x:c r="E15" s="19" t="str"/>
+      <x:c r="F15" s="19" t="str"/>
+      <x:c r="G15" s="19" t="str">
+        <x:v>Local lab only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="19" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B16" s="19" t="str">
+        <x:v>Auth and session security</x:v>
+      </x:c>
+      <x:c r="C16" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D16" s="19" t="str"/>
+      <x:c r="E16" s="19" t="str"/>
+      <x:c r="F16" s="19" t="str"/>
+      <x:c r="G16" s="19" t="str">
+        <x:v>Test accounts only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="19" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="19" t="str">
+        <x:v>Access-control testing</x:v>
+      </x:c>
+      <x:c r="C17" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D17" s="19" t="str"/>
+      <x:c r="E17" s="19" t="str"/>
+      <x:c r="F17" s="19" t="str"/>
+      <x:c r="G17" s="19" t="str">
+        <x:v>Local lab only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="19" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="19" t="str">
+        <x:v>Secure file upload</x:v>
+      </x:c>
+      <x:c r="C18" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D18" s="19" t="str"/>
+      <x:c r="E18" s="19" t="str"/>
+      <x:c r="F18" s="19" t="str"/>
+      <x:c r="G18" s="19" t="str"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="19" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="19" t="str">
+        <x:v>CSRF defenses</x:v>
+      </x:c>
+      <x:c r="C19" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D19" s="19" t="str"/>
+      <x:c r="E19" s="19" t="str"/>
+      <x:c r="F19" s="19" t="str"/>
+      <x:c r="G19" s="19" t="str">
+        <x:v>Local lab only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="19" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="19" t="str">
+        <x:v>Secret detection</x:v>
+      </x:c>
+      <x:c r="C20" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D20" s="19" t="str"/>
+      <x:c r="E20" s="19" t="str"/>
+      <x:c r="F20" s="19" t="str"/>
+      <x:c r="G20" s="19" t="str">
+        <x:v>Synthetic repositories only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="19" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="19" t="str">
+        <x:v>File-integrity monitoring</x:v>
+      </x:c>
+      <x:c r="C21" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D21" s="19" t="str"/>
+      <x:c r="E21" s="19" t="str"/>
+      <x:c r="F21" s="19" t="str"/>
+      <x:c r="G21" s="19" t="str"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="19" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="19" t="str">
+        <x:v>Authentication-log analysis</x:v>
+      </x:c>
+      <x:c r="C22" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D22" s="19" t="str"/>
+      <x:c r="E22" s="19" t="str"/>
+      <x:c r="F22" s="19" t="str"/>
+      <x:c r="G22" s="19" t="str">
+        <x:v>Synthetic logs only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="19" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="19" t="str">
+        <x:v>Windows defensive audit</x:v>
+      </x:c>
+      <x:c r="C23" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D23" s="19" t="str"/>
+      <x:c r="E23" s="19" t="str"/>
+      <x:c r="F23" s="19" t="str"/>
+      <x:c r="G23" s="19" t="str">
+        <x:v>Read-only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="19" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="19" t="str">
+        <x:v>Ports and firewall inventory</x:v>
+      </x:c>
+      <x:c r="C24" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D24" s="19" t="str"/>
+      <x:c r="E24" s="19" t="str"/>
+      <x:c r="F24" s="19" t="str"/>
+      <x:c r="G24" s="19" t="str">
+        <x:v>Local machine only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="19" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B25" s="19" t="str">
+        <x:v>Backup integrity checker</x:v>
+      </x:c>
+      <x:c r="C25" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D25" s="19" t="str"/>
+      <x:c r="E25" s="19" t="str"/>
+      <x:c r="F25" s="19" t="str"/>
+      <x:c r="G25" s="19" t="str">
+        <x:v>Test data</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="19" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B26" s="19" t="str">
+        <x:v>Rate-limit simulator</x:v>
+      </x:c>
+      <x:c r="C26" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D26" s="19" t="str"/>
+      <x:c r="E26" s="19" t="str"/>
+      <x:c r="F26" s="19" t="str"/>
+      <x:c r="G26" s="19" t="str">
+        <x:v>Local mock service</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="19" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B27" s="19" t="str">
+        <x:v>Bot-abuse simulator</x:v>
+      </x:c>
+      <x:c r="C27" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D27" s="19" t="str"/>
+      <x:c r="E27" s="19" t="str"/>
+      <x:c r="F27" s="19" t="str"/>
+      <x:c r="G27" s="19" t="str">
+        <x:v>Local mock service</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="19" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B28" s="19" t="str">
+        <x:v>Incident response playbook</x:v>
+      </x:c>
+      <x:c r="C28" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D28" s="19" t="str"/>
+      <x:c r="E28" s="19" t="str"/>
+      <x:c r="F28" s="19" t="str"/>
+      <x:c r="G28" s="19" t="str">
+        <x:v>Synthetic incident</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="19" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B29" s="19" t="str">
+        <x:v>Threat model</x:v>
+      </x:c>
+      <x:c r="C29" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D29" s="19" t="str"/>
+      <x:c r="E29" s="19" t="str"/>
+      <x:c r="F29" s="19" t="str"/>
+      <x:c r="G29" s="19" t="str">
+        <x:v>Sample app</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="19" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B30" s="19" t="str">
+        <x:v>Cybersecurity dashboard</x:v>
+      </x:c>
+      <x:c r="C30" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D30" s="19" t="str"/>
+      <x:c r="E30" s="19" t="str"/>
+      <x:c r="F30" s="19" t="str"/>
+      <x:c r="G30" s="19" t="str">
+        <x:v>Generated/sample data</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="19" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B31" s="19" t="str">
+        <x:v>OWASP ZAP baseline</x:v>
+      </x:c>
+      <x:c r="C31" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D31" s="19" t="str"/>
+      <x:c r="E31" s="19" t="str"/>
+      <x:c r="F31" s="19" t="str"/>
+      <x:c r="G31" s="19" t="str">
+        <x:v>Local training app or authorized target only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="19" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B32" s="19" t="str">
+        <x:v>Fix and retest</x:v>
+      </x:c>
+      <x:c r="C32" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D32" s="19" t="str"/>
+      <x:c r="E32" s="19" t="str"/>
+      <x:c r="F32" s="19" t="str"/>
+      <x:c r="G32" s="19" t="str"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="19" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B33" s="19" t="str">
+        <x:v>Portfolio consolidation</x:v>
+      </x:c>
+      <x:c r="C33" s="19" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+      <x:c r="D33" s="19" t="str"/>
+      <x:c r="E33" s="19" t="str"/>
+      <x:c r="F33" s="19" t="str"/>
+      <x:c r="G33" s="19" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="38" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="9" t="str">
+        <x:v>Tools Used — Verified for Day 1</x:v>
+      </x:c>
+      <x:c r="B1" s="9" t="str"/>
+      <x:c r="C1" s="9" t="str"/>
+      <x:c r="D1" s="9" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="20" t="str">
+        <x:v>Tool</x:v>
+      </x:c>
+      <x:c r="B3" s="20" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="C3" s="20" t="str">
+        <x:v>Observed status/version</x:v>
+      </x:c>
+      <x:c r="D3" s="20" t="str">
+        <x:v>Used in</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="19" t="str">
+        <x:v>OpenClaw</x:v>
+      </x:c>
+      <x:c r="B4" s="19" t="str">
+        <x:v>Orchestration and scheduled agent workflow</x:v>
+      </x:c>
+      <x:c r="C4" s="19" t="str">
+        <x:v>Installed; exact version not captured</x:v>
+      </x:c>
+      <x:c r="D4" s="19" t="str">
+        <x:v>Project system</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="19" t="str">
+        <x:v>Ollama</x:v>
+      </x:c>
+      <x:c r="B5" s="19" t="str">
+        <x:v>Local model runtime</x:v>
+      </x:c>
+      <x:c r="C5" s="19" t="str">
+        <x:v>Available; qwen3:4b listed</x:v>
+      </x:c>
+      <x:c r="D5" s="19" t="str">
+        <x:v>Local AI analysis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="19" t="str">
+        <x:v>Qwen3:4B</x:v>
+      </x:c>
+      <x:c r="B6" s="19" t="str">
+        <x:v>Local AI model</x:v>
+      </x:c>
+      <x:c r="C6" s="19" t="str">
+        <x:v>Installed in Ollama</x:v>
+      </x:c>
+      <x:c r="D6" s="19" t="str">
+        <x:v>Required model</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="19" t="str">
+        <x:v>Python</x:v>
+      </x:c>
+      <x:c r="B7" s="19" t="str">
+        <x:v>Automation and tests</x:v>
+      </x:c>
+      <x:c r="C7" s="19" t="str">
+        <x:v>3.13.14</x:v>
+      </x:c>
+      <x:c r="D7" s="19" t="str">
+        <x:v>Day 1 verifier and future utilities</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="19" t="str">
+        <x:v>Git</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="str">
+        <x:v>Version control</x:v>
+      </x:c>
+      <x:c r="C8" s="19" t="str">
+        <x:v>2.55.0.windows.3</x:v>
+      </x:c>
+      <x:c r="D8" s="19" t="str">
+        <x:v>Portfolio history and GitHub upload</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="19" t="str">
+        <x:v>PowerShell</x:v>
+      </x:c>
+      <x:c r="B9" s="19" t="str">
+        <x:v>Windows-compatible setup and file operations</x:v>
+      </x:c>
+      <x:c r="C9" s="19" t="str">
+        <x:v>Available</x:v>
+      </x:c>
+      <x:c r="D9" s="19" t="str">
+        <x:v>Environment setup</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="19" t="str">
+        <x:v>curl</x:v>
+      </x:c>
+      <x:c r="B10" s="19" t="str">
+        <x:v>Free HTTP/TLS utility</x:v>
+      </x:c>
+      <x:c r="C10" s="19" t="str">
+        <x:v>8.21.0</x:v>
+      </x:c>
+      <x:c r="D10" s="19" t="str">
+        <x:v>Available for authorized/local checks</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="19" t="str">
+        <x:v>GitHub CLI</x:v>
+      </x:c>
+      <x:c r="B11" s="19" t="str">
+        <x:v>Repository creation and upload</x:v>
+      </x:c>
+      <x:c r="C11" s="19" t="str">
+        <x:v>Authenticated as amalraj020-a11y</x:v>
+      </x:c>
+      <x:c r="D11" s="19" t="str">
+        <x:v>Portfolio upload</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="19" t="str">
+        <x:v>Codex Artifact Tool</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="str">
+        <x:v>Excel workbook creation/editing</x:v>
+      </x:c>
+      <x:c r="C12" s="19" t="str">
+        <x:v>Bundled runtime</x:v>
+      </x:c>
+      <x:c r="D12" s="19" t="str">
+        <x:v>This workbook</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:D1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>